<commit_message>
Split Sego CZ26007736 HS summary into invoiced and FOC shipments
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHCMC3ZGrhkK1VPceYbSSc
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sego_CZ26007736.xlsx
+++ b/output/HS_Code_Summary_Sego_CZ26007736.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,15 +37,27 @@
       <color rgb="009C0006"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
       <color rgb="009C0006"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -76,11 +88,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -88,10 +102,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -462,10 +476,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -578,278 +592,431 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>HS kód</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Popis</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Netto (kg)</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Brutto (kg)</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Množství (ks)</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Celní hodnota (RMB)</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Antidumping</t>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Deklarace:</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>ROZDĚLENO NA 2 ZÁSILKY – 1) fakturované zboží, 2) položky FOC (zdarma)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>ZÁSILKA 1 – FAKTUROVANÉ ZBOŽÍ (faktura 26ZMKA038 – 193 863,80 RMB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>HS kód</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Popis</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Netto (kg)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Brutto (kg)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Množství (ks)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Celní hodnota (RMB)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Antidumping</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>9401 30 00</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Kancelářské otočné židle, výškově nastavitelné (Stretch New, Greny, Pixel, Sky G)</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C15" s="8" t="n">
         <v>6714.1</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D15" s="8" t="n">
         <v>7721.2</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E15" s="6" t="n">
         <v>393</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F15" s="8" t="n">
         <v>193143.8</v>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Ne – ověřit TARIC</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>9401 90 80</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Náhradní díly židlí – pětiramenný kříž, plastové kryty sedáku, kompletní opěrák Stretch New</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>92.5</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>1260</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Náhradní díl židlí – pětiramenný kříž nylon (Pixel)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>720</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Ne – ověřit TARIC</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>CELKEM</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n">
+        <v>6774.1</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>7784.2</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>423</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>193863.8</v>
+      </c>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ZÁSILKA 2 – POLOŽKY FOC / ZDARMA (hodnota dle VDD – 996,15 RMB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>HS kód</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Popis</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Netto (kg)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Brutto (kg)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Množství (ks)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Celní hodnota (RMB)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Antidumping</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>9401 90 80</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Náhradní díly židlí FOC – plastové kryty sedáku (Simple New, Stretch New, Cool), kompletní opěrák Stretch New</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>540</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Ne</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Ne – ověřit TARIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>9401 99 10</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Náhradní díly židlí – plynové písty (Stretch, Spirit, Ego), synchronní mechanika Tecton</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Náhradní díly židlí FOC – plynové písty (Stretch, Spirit, Ego), synchronní mechanika Tecton</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D22" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F22" s="8" t="n">
         <v>456.15</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Ne – ověřit TARIC</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="8" t="n">
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="10" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>996.15</v>
+      </c>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>KONTROLNÍ SOUČET OBĚ ZÁSILKY</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="10" t="n">
         <v>6836.6</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D25" s="10" t="n">
         <v>7852.7</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E25" s="9" t="n">
         <v>457</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F25" s="10" t="n">
         <v>194859.95</v>
       </c>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    </row>
+    <row r="26">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>odpovídá packing listu (457 ks / 6 836,6 kg / 7 852,7 kg / 405 CTNS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>⚠️ PREFERENČNÍ VĚTA:</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>V dokladech (faktura 26ZMKA038, B/L F202614540) NENÍ uvedena žádná preferenční věta. Původ Čína – EU nemá s Čínou preferenční dohodu, uplatní se standardní všeobecná/třetizemní sazba cla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Hodnota:</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Fakturovaná hodnota 193 863,80 RMB + neocenené náhradní díly FOC vyčíslené ve VDD na 996,15 RMB = celní hodnota celkem 194 859,95 RMB. FOC položky: 9401 99 10 celé (456,15 RMB) a část 9401 90 80 (540,00 RMB).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>V dokladech (faktura 26ZMKA038, B/L F202614540) NENÍ uvedena žádná preferenční věta. Původ Čína – EU nemá s Čínou preferenční dohodu, uplatní se standardní třetizemní sazba cla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ FOC / 2 zásilky:</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Faktura obsahuje položky FOC (řádky 6–13 CI, cena 0). Deklarace bude rozdělena na 2 zásilky: zásilka 1 = fakturované zboží (193 863,80 RMB), zásilka 2 = FOC položky oceněné dle VDD (996,15 RMB). Pozn.: HS 9401 90 80 se vyskytuje v obou zásilkách.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Váhy FOC položek:</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Písty Spirit/Ego a kryt sedáku Cool nemají v packing listu samostatnou váhu – jsou baleny v kartonech sousedních položek stejného HS kódu, váhy per HS kód proto sedí na celkové NW 6 836,6 / GW 7 852,7 kg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Písty Spirit/Ego jsou baleny v kartonu s pístem Stretch a kryt Cool v kartonu s krytem Stretch New (vše FOC, stejné HS) – váhy per HS kód i rozdělení na zásilky proto sedí na celkové NW 6 836,6 / GW 7 852,7 kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>HS kódy – upozornění:</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>Kód 9401 30 00 z VDD je od HS 2022 zrušen (rozdělen na 9401 31 00 dřevěná / 9401 39 00 ostatní) – tyto židle patrně patří pod 9401 39 00. Kód 9401 90 80 je rovněž starý (nyní 9401 91/9401 99); 9401 99 10 je dle aktuální CN určen pro díly sedadel letadel – pro díly kancelářských židlí ověřit 9401 99 80. Doporučuji ověřit v TARIC před podáním JSD.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Antidumping:</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>K datu zpracování nebylo dohledáno platné antidumpingové opatření EU na kancelářské židle (HS 9401) z Číny – doporučuji ověřit aktuální stav v TARIC při propuštění.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>CBAM:</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Zboží (sedadla a jejich díly, kap. 94) nespadá pod CBAM.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Sleva:</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Faktura neobsahuje žádnou obchodní slevu – žádné rozpočítání se neuplatní.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Y kódy:</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Dle pokynu ignorovány – budou dodány později.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B23:H23"/>
+  <mergeCells count="10">
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="B28:H28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>